<commit_message>
Update common detailed design and align menu contracts
</commit_message>
<xml_diff>
--- a/基本設計/02_権限基本設計書.xlsx
+++ b/基本設計/02_権限基本設計書.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_表紙" sheetId="1" r:id="R51d1f6bed6674a93"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_改訂履歴" sheetId="2" r:id="Rb903e54b68224279"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_ロール定義" sheetId="10" r:id="Rd120777407f94afc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_メニュー権限" sheetId="11" r:id="R704dfdf16c73452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_機能権限" sheetId="12" r:id="Rc5d3d8f041de4ce0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_権限コード" sheetId="13" r:id="R5072afd4190048ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_API権限対応" sheetId="14" r:id="R58d5e3ab94234d99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_DataScope定義" sheetId="15" r:id="R6d6d49eeaeb9461f"/>
-  </x:sheets>
-</x:workbook>
+<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <ns0:sheets>
+    <ns0:sheet name="00_表紙" sheetId="1" ns1:id="Red7a016096414262"/>
+    <ns0:sheet name="01_改訂履歴" sheetId="2" ns1:id="R22a2339b2a494254"/>
+    <ns0:sheet name="09_ロール定義" sheetId="10" ns1:id="R8a31b0ab31dd4e69"/>
+    <ns0:sheet name="10_メニュー権限" sheetId="11" ns1:id="R127af4c83c3e4088"/>
+    <ns0:sheet name="11_機能権限" sheetId="12" ns1:id="R6fba5db5a05e43ed"/>
+    <ns0:sheet name="12_権限コード" sheetId="13" ns1:id="R4f48ac6dba5a4439"/>
+    <ns0:sheet name="13_API権限対応" sheetId="14" ns1:id="R2812ea5abce04dd9"/>
+    <ns0:sheet name="14_DataScope定義" sheetId="15" ns1:id="R73c5b748e74d4ce8"/>
+  </ns0:sheets>
+</ns0:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -23,7 +23,7 @@
   <x:numFmts count="1">
     <x:numFmt numFmtId="200" formatCode="yyyy-mm-dd"/>
   </x:numFmts>
-  <x:fonts count="27">
+  <x:fonts count="28">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -173,8 +173,13 @@
       <x:color rgb="FF193C61"/>
       <x:name val="Yu Gothic"/>
     </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF17212B"/>
+      <x:name val="Yu Gothic"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="31">
+  <x:fills count="34">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -326,6 +331,21 @@
         <x:fgColor rgb="FFF1F5FA"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF1F4E78"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEDF3F8"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
   <x:borders count="9">
     <x:border/>
@@ -403,7 +423,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="254">
+  <x:cellXfs count="264">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -940,6 +960,26 @@
       <x:alignment vertical="top" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="12" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="32" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="27" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="27" fillId="33" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="top" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="31" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
     <x:cellStyle name="Normal" xfId="0"/>
@@ -1387,7 +1427,7 @@
       <x:c r="A11"/>
       <x:c r="B11"/>
       <x:c r="C11" s="235" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="D11"/>
       <x:c r="E11"/>
@@ -1424,7 +1464,7 @@
         <x:v>版数</x:v>
       </x:c>
       <x:c r="D13" s="238" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="E13" s="191"/>
       <x:c r="F13" s="191"/>
@@ -1442,7 +1482,7 @@
         <x:v>改訂日</x:v>
       </x:c>
       <x:c r="D14" s="238" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="E14" s="191"/>
       <x:c r="F14" s="191"/>
@@ -1478,7 +1518,7 @@
         <x:v>状態</x:v>
       </x:c>
       <x:c r="D16" s="238" t="str">
-        <x:v>Review中</x:v>
+        <x:v>修正済</x:v>
       </x:c>
       <x:c r="E16" s="191"/>
       <x:c r="F16" s="191"/>
@@ -1639,7 +1679,7 @@
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
       <x:c r="A4" s="244" t="str">
-        <x:v>版数：Ver.2.5    改訂日：2026-09-24    Baseline：BL-2026-09-24</x:v>
+        <x:v>版数：Ver.2.6    改訂日：2026-09-29    Baseline：BL-2026-09-24</x:v>
       </x:c>
       <x:c r="B4" s="63"/>
       <x:c r="C4" s="63"/>
@@ -2115,6 +2155,32 @@
       </x:c>
       <x:c r="H21" s="240" t="str">
         <x:v>BL-2026-09-24。責任者・Review者・承認者はProject Leaderが記入。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="22" ht="95" customHeight="1">
+      <x:c r="A22" t="str">
+        <x:v>Ver.2.6</x:v>
+      </x:c>
+      <x:c r="B22" t="str">
+        <x:v>2026-09-29</x:v>
+      </x:c>
+      <x:c r="C22" t="str">
+        <x:v>CHG-MENU-20260929-01：U-01対応。固定Menu Code・menus契約・下流Bindingを整合。既存権限・Route・DBは変更なし。</x:v>
+      </x:c>
+      <x:c r="D22" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="E22" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F22" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="G22" t="str">
+        <x:v>修正済</x:v>
+      </x:c>
+      <x:c r="H22" t="str">
+        <x:v>方式合意に基づく補完。成果物の正式承認は別途。</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -2199,7 +2265,7 @@
       </x:c>
       <x:c r="B4" s="23"/>
       <x:c r="C4" s="242" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="D4" s="21"/>
       <x:c r="E4" s="23" t="str">
@@ -2207,7 +2273,7 @@
       </x:c>
       <x:c r="F4" s="23"/>
       <x:c r="G4" s="243" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="H4"/>
       <x:c r="I4"/>
@@ -2562,11 +2628,11 @@
       </x:c>
       <x:c r="B4" s="23"/>
       <x:c r="C4" s="242" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="D4" s="21"/>
       <x:c r="E4" s="241" t="str">
-        <x:v>作成日：2026-09-24</x:v>
+        <x:v>作成日：2026-09-29</x:v>
       </x:c>
       <x:c r="F4" s="35"/>
       <x:c r="G4" s="36"/>
@@ -2980,6 +3046,466 @@
       </x:c>
       <x:c r="F22" s="33" t="str"/>
     </x:row>
+    <x:row r="25" ht="30" customHeight="1">
+      <x:c r="A25" s="255" t="str">
+        <x:v>2. Menu Code定義（API-AUTH-004 menus正本）</x:v>
+      </x:c>
+      <x:c r="B25" s="255"/>
+      <x:c r="C25" s="255"/>
+      <x:c r="D25" s="255"/>
+      <x:c r="E25" s="255"/>
+      <x:c r="F25" s="255"/>
+    </x:row>
+    <x:row r="26" ht="30" customHeight="1">
+      <x:c r="A26" s="263" t="str">
+        <x:v>Menu Code</x:v>
+      </x:c>
+      <x:c r="B26" s="263" t="str">
+        <x:v>表示名（上表参照）</x:v>
+      </x:c>
+      <x:c r="C26" s="263" t="str">
+        <x:v>画面ID</x:v>
+      </x:c>
+      <x:c r="D26" s="263" t="str">
+        <x:v>表示順</x:v>
+      </x:c>
+      <x:c r="E26" s="263" t="str">
+        <x:v>固定Query</x:v>
+      </x:c>
+      <x:c r="F26" s="263" t="str">
+        <x:v>権限参照</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27" ht="42" customHeight="1">
+      <x:c r="A27" s="259" t="str">
+        <x:v>MENU-HOME</x:v>
+      </x:c>
+      <x:c r="B27" s="259" t="str">
+        <x:v>ダッシュボード</x:v>
+      </x:c>
+      <x:c r="C27" s="259" t="str">
+        <x:v>SCR-002</x:v>
+      </x:c>
+      <x:c r="D27" s="259" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="E27" s="259" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F27" s="259" t="str">
+        <x:v>本Sheet行8のRole条件。認証済共通。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28" ht="42" customHeight="1">
+      <x:c r="A28" s="262" t="str">
+        <x:v>MENU-EMPLOYEES</x:v>
+      </x:c>
+      <x:c r="B28" s="262" t="str">
+        <x:v>従業員管理</x:v>
+      </x:c>
+      <x:c r="C28" s="262" t="str">
+        <x:v>SCR-003</x:v>
+      </x:c>
+      <x:c r="D28" s="262" t="n">
+        <x:v>2</x:v>
+      </x:c>
+      <x:c r="E28" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F28" s="262" t="str">
+        <x:v>本Sheet行9のRole条件。PERM-EMP-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29" ht="42" customHeight="1">
+      <x:c r="A29" s="259" t="str">
+        <x:v>MENU-DEPARTMENTS</x:v>
+      </x:c>
+      <x:c r="B29" s="259" t="str">
+        <x:v>部門管理</x:v>
+      </x:c>
+      <x:c r="C29" s="259" t="str">
+        <x:v>SCR-007</x:v>
+      </x:c>
+      <x:c r="D29" s="259" t="n">
+        <x:v>3</x:v>
+      </x:c>
+      <x:c r="E29" s="259" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F29" s="259" t="str">
+        <x:v>本Sheet行10のRole条件。PERM-DEPT-WRITE（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30" ht="42" customHeight="1">
+      <x:c r="A30" s="262" t="str">
+        <x:v>MENU-PROJECTS</x:v>
+      </x:c>
+      <x:c r="B30" s="262" t="str">
+        <x:v>プロジェクト一覧</x:v>
+      </x:c>
+      <x:c r="C30" s="262" t="str">
+        <x:v>SCR-008</x:v>
+      </x:c>
+      <x:c r="D30" s="262" t="n">
+        <x:v>4</x:v>
+      </x:c>
+      <x:c r="E30" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F30" s="262" t="str">
+        <x:v>本Sheet行11のRole条件。PERM-PRJ-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31" ht="42" customHeight="1">
+      <x:c r="A31" s="259" t="str">
+        <x:v>MENU-MY-PROJECTS</x:v>
+      </x:c>
+      <x:c r="B31" s="259" t="str">
+        <x:v>マイプロジェクト</x:v>
+      </x:c>
+      <x:c r="C31" s="259" t="str">
+        <x:v>SCR-008</x:v>
+      </x:c>
+      <x:c r="D31" s="259" t="n">
+        <x:v>5</x:v>
+      </x:c>
+      <x:c r="E31" s="259" t="str">
+        <x:v>mine=true</x:v>
+      </x:c>
+      <x:c r="F31" s="259" t="str">
+        <x:v>本Sheet行12のRole条件。PERM-PRJ-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32" ht="42" customHeight="1">
+      <x:c r="A32" s="262" t="str">
+        <x:v>MENU-TASKS</x:v>
+      </x:c>
+      <x:c r="B32" s="262" t="str">
+        <x:v>全タスク</x:v>
+      </x:c>
+      <x:c r="C32" s="262" t="str">
+        <x:v>SCR-013</x:v>
+      </x:c>
+      <x:c r="D32" s="262" t="n">
+        <x:v>6</x:v>
+      </x:c>
+      <x:c r="E32" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F32" s="262" t="str">
+        <x:v>本Sheet行13のRole条件。PERM-TASK-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="33" ht="42" customHeight="1">
+      <x:c r="A33" s="259" t="str">
+        <x:v>MENU-MY-TASKS</x:v>
+      </x:c>
+      <x:c r="B33" s="259" t="str">
+        <x:v>マイタスク</x:v>
+      </x:c>
+      <x:c r="C33" s="259" t="str">
+        <x:v>SCR-014</x:v>
+      </x:c>
+      <x:c r="D33" s="259" t="n">
+        <x:v>7</x:v>
+      </x:c>
+      <x:c r="E33" s="259" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F33" s="259" t="str">
+        <x:v>本Sheet行14のRole条件。PERM-TASK-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="34" ht="42" customHeight="1">
+      <x:c r="A34" s="262" t="str">
+        <x:v>MENU-TASK-BOARD</x:v>
+      </x:c>
+      <x:c r="B34" s="262" t="str">
+        <x:v>タスクボード</x:v>
+      </x:c>
+      <x:c r="C34" s="262" t="str">
+        <x:v>SCR-018</x:v>
+      </x:c>
+      <x:c r="D34" s="262" t="n">
+        <x:v>8</x:v>
+      </x:c>
+      <x:c r="E34" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F34" s="262" t="str">
+        <x:v>本Sheet行15のRole条件。PERM-TASK-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35" ht="42" customHeight="1">
+      <x:c r="A35" s="259" t="str">
+        <x:v>MENU-MY-REPORTS</x:v>
+      </x:c>
+      <x:c r="B35" s="259" t="str">
+        <x:v>マイ日報</x:v>
+      </x:c>
+      <x:c r="C35" s="259" t="str">
+        <x:v>SCR-019</x:v>
+      </x:c>
+      <x:c r="D35" s="259" t="n">
+        <x:v>9</x:v>
+      </x:c>
+      <x:c r="E35" s="259" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F35" s="259" t="str">
+        <x:v>本Sheet行16のRole条件。PERM-RPT-SELF（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36" ht="42" customHeight="1">
+      <x:c r="A36" s="262" t="str">
+        <x:v>MENU-REPORT-SEARCH</x:v>
+      </x:c>
+      <x:c r="B36" s="262" t="str">
+        <x:v>日報検索</x:v>
+      </x:c>
+      <x:c r="C36" s="262" t="str">
+        <x:v>SCR-021</x:v>
+      </x:c>
+      <x:c r="D36" s="262" t="n">
+        <x:v>10</x:v>
+      </x:c>
+      <x:c r="E36" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F36" s="262" t="str">
+        <x:v>本Sheet行17のRole条件。PERM-RPT-TEAM（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37" ht="42" customHeight="1">
+      <x:c r="A37" s="259" t="str">
+        <x:v>MENU-NOTIFICATIONS</x:v>
+      </x:c>
+      <x:c r="B37" s="259" t="str">
+        <x:v>通知一覧</x:v>
+      </x:c>
+      <x:c r="C37" s="259" t="str">
+        <x:v>SCR-022</x:v>
+      </x:c>
+      <x:c r="D37" s="259" t="n">
+        <x:v>11</x:v>
+      </x:c>
+      <x:c r="E37" s="259" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F37" s="259" t="str">
+        <x:v>本Sheet行19のRole条件。認証済共通。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38" ht="42" customHeight="1">
+      <x:c r="A38" s="262" t="str">
+        <x:v>MENU-USERS</x:v>
+      </x:c>
+      <x:c r="B38" s="262" t="str">
+        <x:v>ユーザー管理</x:v>
+      </x:c>
+      <x:c r="C38" s="262" t="str">
+        <x:v>SCR-023</x:v>
+      </x:c>
+      <x:c r="D38" s="262" t="n">
+        <x:v>12</x:v>
+      </x:c>
+      <x:c r="E38" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F38" s="262" t="str">
+        <x:v>本Sheet行20のRole条件。PERM-USER-ADMIN（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39" ht="42" customHeight="1">
+      <x:c r="A39" s="259" t="str">
+        <x:v>MENU-ROLES</x:v>
+      </x:c>
+      <x:c r="B39" s="259" t="str">
+        <x:v>ロール/権限</x:v>
+      </x:c>
+      <x:c r="C39" s="259" t="str">
+        <x:v>SCR-024</x:v>
+      </x:c>
+      <x:c r="D39" s="259" t="n">
+        <x:v>13</x:v>
+      </x:c>
+      <x:c r="E39" s="259" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F39" s="259" t="str">
+        <x:v>本Sheet行21のRole条件。PERM-ROLE-ADMIN（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40" ht="42" customHeight="1">
+      <x:c r="A40" s="262" t="str">
+        <x:v>MENU-LOGS</x:v>
+      </x:c>
+      <x:c r="B40" s="262" t="str">
+        <x:v>操作ログ</x:v>
+      </x:c>
+      <x:c r="C40" s="262" t="str">
+        <x:v>SCR-025</x:v>
+      </x:c>
+      <x:c r="D40" s="262" t="n">
+        <x:v>14</x:v>
+      </x:c>
+      <x:c r="E40" s="262" t="str">
+        <x:v>－</x:v>
+      </x:c>
+      <x:c r="F40" s="262" t="str">
+        <x:v>本Sheet行22のRole条件。PERM-LOG-READ（12参照）。Data Scopeは13・14参照。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="30" customHeight="1">
+      <x:c r="A44" s="255" t="str">
+        <x:v>3. Menu生成・利用規則</x:v>
+      </x:c>
+      <x:c r="B44" s="255"/>
+      <x:c r="C44" s="255"/>
+      <x:c r="D44" s="255"/>
+      <x:c r="E44" s="255"/>
+      <x:c r="F44" s="255"/>
+    </x:row>
+    <x:row r="45" ht="30" customHeight="1">
+      <x:c r="A45" s="263" t="str">
+        <x:v>項目</x:v>
+      </x:c>
+      <x:c r="B45" s="263" t="str">
+        <x:v>定義</x:v>
+      </x:c>
+      <x:c r="C45" s="263" t="str">
+        <x:v>参照</x:v>
+      </x:c>
+      <x:c r="D45" s="263" t="str">
+        <x:v>対象</x:v>
+      </x:c>
+      <x:c r="E45" s="263" t="str">
+        <x:v>条件</x:v>
+      </x:c>
+      <x:c r="F45" s="263" t="str">
+        <x:v>補足</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="57" customHeight="1">
+      <x:c r="A46" s="259" t="str">
+        <x:v>識別値</x:v>
+      </x:c>
+      <x:c r="B46" s="259" t="str">
+        <x:v>Menu Codeは表示名ではなく固定識別子。大文字小文字を区別し、部分一致・Trim変換をしない。</x:v>
+      </x:c>
+      <x:c r="C46" s="259" t="str">
+        <x:v>本Sheet2節</x:v>
+      </x:c>
+      <x:c r="D46" s="259" t="str">
+        <x:v>API-AUTH-004</x:v>
+      </x:c>
+      <x:c r="E46" s="259" t="str">
+        <x:v>第1期14 Menu</x:v>
+      </x:c>
+      <x:c r="F46" s="259" t="str">
+        <x:v>親見出しは返却しない。日報統計（行18）は第1期非提供のためCodeを追加・返却しない。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="57" customHeight="1">
+      <x:c r="A47" s="262" t="str">
+        <x:v>表示候補</x:v>
+      </x:c>
+      <x:c r="B47" s="262" t="str">
+        <x:v>有効Roleの上表許可を和集合にし、必要Permissionと積集合。表示順の昇順で重複なしのCode配列を返す。</x:v>
+      </x:c>
+      <x:c r="C47" s="262" t="str">
+        <x:v>09・12／本Sheet1・2節</x:v>
+      </x:c>
+      <x:c r="D47" s="262" t="str">
+        <x:v>roles / permissions / menus</x:v>
+      </x:c>
+      <x:c r="E47" s="262" t="str">
+        <x:v>未許可Menuは返さない</x:v>
+      </x:c>
+      <x:c r="F47" s="262" t="str">
+        <x:v>Role・Data Scopeを拡張しない。Homeは共通安全画面。Dashboard集計APIのPERM-DASH-READは別判定。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="57" customHeight="1">
+      <x:c r="A48" s="259" t="str">
+        <x:v>空配列</x:v>
+      </x:c>
+      <x:c r="B48" s="259" t="str">
+        <x:v>menus=[]は許容する。ClientはMenuを自動補完せず、空の親見出しも表示しない。</x:v>
+      </x:c>
+      <x:c r="C48" s="259" t="str">
+        <x:v>10／23_API項目定義</x:v>
+      </x:c>
+      <x:c r="D48" s="259" t="str">
+        <x:v>Menu表示</x:v>
+      </x:c>
+      <x:c r="E48" s="259" t="str">
+        <x:v>Null・Null要素不可</x:v>
+      </x:c>
+      <x:c r="F48" s="259" t="str">
+        <x:v>通常の組込Role利用者は上表により表示候補を持つ。空配列の許容は権限拡張を意味しない。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="42" customHeight="1">
+      <x:c r="A49" s="262" t="str">
+        <x:v>画面遷移</x:v>
+      </x:c>
+      <x:c r="B49" s="262" t="str">
+        <x:v>画面IDのPathは03のRoute定義を参照。固定Queryは2節による。</x:v>
+      </x:c>
+      <x:c r="C49" s="262" t="str">
+        <x:v>03／20_画面Route定義</x:v>
+      </x:c>
+      <x:c r="D49" s="262" t="str">
+        <x:v>各Menu選択</x:v>
+      </x:c>
+      <x:c r="E49" s="262" t="str">
+        <x:v>遷移前にGuardを実行</x:v>
+      </x:c>
+      <x:c r="F49" s="262" t="str">
+        <x:v>マイプロジェクトはSCR-008にmine=trueを付ける。親見出しにリンクを設定しない。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="57" customHeight="1">
+      <x:c r="A50" s="259" t="str">
+        <x:v>Client防御</x:v>
+      </x:c>
+      <x:c r="B50" s="259" t="str">
+        <x:v>未知の文字列Codeは無視しリンク化しない。重複Codeは表示時に1件へ集約する。</x:v>
+      </x:c>
+      <x:c r="C50" s="259" t="str">
+        <x:v>10／23_API項目定義</x:v>
+      </x:c>
+      <x:c r="D50" s="259" t="str">
+        <x:v>Menu構築</x:v>
+      </x:c>
+      <x:c r="E50" s="259" t="str">
+        <x:v>CodeをURL・HTMLとして使用しない</x:v>
+      </x:c>
+      <x:c r="F50" s="259" t="str">
+        <x:v>Serverは2節のCodeのみ・重複なしを保証。Clientの防御は契約外の値を正規Codeと認めるものではない。</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="42" customHeight="1">
+      <x:c r="A51" s="262" t="str">
+        <x:v>強制改密</x:v>
+      </x:c>
+      <x:c r="B51" s="262" t="str">
+        <x:v>passwordMustChange=trueの表示・遷移制限は既定Guardに従う。</x:v>
+      </x:c>
+      <x:c r="C51" s="262" t="str">
+        <x:v>03／20_画面Route定義</x:v>
+      </x:c>
+      <x:c r="D51" s="262" t="str">
+        <x:v>SCR-026</x:v>
+      </x:c>
+      <x:c r="E51" s="262" t="str">
+        <x:v>通常Menuを表示しない</x:v>
+      </x:c>
+      <x:c r="F51" s="262" t="str">
+        <x:v>menus生成で既存Role/Permissionを変更しない。画面・APIの最終認可はMenu表示とは別に実施する。</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:mergeCells>
     <x:mergeCell ref="A1:F2"/>
@@ -2991,6 +3517,8 @@
     <x:mergeCell ref="C4:D4"/>
     <x:mergeCell ref="A6:F6"/>
     <x:mergeCell ref="E4:G4"/>
+    <x:mergeCell ref="A25:F25"/>
+    <x:mergeCell ref="A44:F44"/>
   </x:mergeCells>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -3067,7 +3595,7 @@
       </x:c>
       <x:c r="B4" s="23"/>
       <x:c r="C4" s="242" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="D4" s="21"/>
       <x:c r="E4" s="23" t="str">
@@ -3075,7 +3603,7 @@
       </x:c>
       <x:c r="F4" s="23"/>
       <x:c r="G4" s="243" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="H4"/>
       <x:c r="I4"/>
@@ -3708,13 +4236,13 @@
         <x:v>版数</x:v>
       </x:c>
       <x:c r="B4" s="63" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="C4" s="62" t="str">
         <x:v>改訂日</x:v>
       </x:c>
       <x:c r="D4" s="63" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="E4" s="63"/>
       <x:c r="F4" s="63"/>
@@ -4281,14 +4809,14 @@
         <x:v>版数</x:v>
       </x:c>
       <x:c r="B4" s="63" t="str">
-        <x:v>Ver.2.5</x:v>
+        <x:v>Ver.2.6</x:v>
       </x:c>
       <x:c r="C4" s="139"/>
       <x:c r="D4" s="141" t="str">
         <x:v>改訂日</x:v>
       </x:c>
       <x:c r="E4" s="63" t="str">
-        <x:v>2026-09-24</x:v>
+        <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="F4" s="139"/>
       <x:c r="G4" s="139"/>

</xml_diff>

<commit_message>
Finalize reviewed menu contract and common frontend design
</commit_message>
<xml_diff>
--- a/基本設計/02_権限基本設計書.xlsx
+++ b/基本設計/02_権限基本設計書.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<ns0:workbook xmlns:ns0="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns1="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <ns0:sheets>
-    <ns0:sheet name="00_表紙" sheetId="1" ns1:id="Red7a016096414262"/>
-    <ns0:sheet name="01_改訂履歴" sheetId="2" ns1:id="R22a2339b2a494254"/>
-    <ns0:sheet name="09_ロール定義" sheetId="10" ns1:id="R8a31b0ab31dd4e69"/>
-    <ns0:sheet name="10_メニュー権限" sheetId="11" ns1:id="R127af4c83c3e4088"/>
-    <ns0:sheet name="11_機能権限" sheetId="12" ns1:id="R6fba5db5a05e43ed"/>
-    <ns0:sheet name="12_権限コード" sheetId="13" ns1:id="R4f48ac6dba5a4439"/>
-    <ns0:sheet name="13_API権限対応" sheetId="14" ns1:id="R2812ea5abce04dd9"/>
-    <ns0:sheet name="14_DataScope定義" sheetId="15" ns1:id="R73c5b748e74d4ce8"/>
-  </ns0:sheets>
-</ns0:workbook>
+<x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheets>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="00_表紙" sheetId="1" r:id="R7728b4bf12e74352"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="01_改訂履歴" sheetId="2" r:id="Rac74ab5c151a400f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_ロール定義" sheetId="10" r:id="R6f6f1215829b4c10"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_メニュー権限" sheetId="11" r:id="Rb6f9b9e03ec04f18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_機能権限" sheetId="12" r:id="R4ba298b69da74d42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_権限コード" sheetId="13" r:id="Rb4dd9d762fb84365"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="13_API権限対応" sheetId="14" r:id="R7bec95dd6aab47c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="14_DataScope定義" sheetId="15" r:id="R068cbfe117d64e91"/>
+  </x:sheets>
+</x:workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2165,7 +2165,7 @@
         <x:v>2026-09-29</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>CHG-MENU-20260929-01：U-01対応。固定Menu Code・menus契約・下流Bindingを整合。既存権限・Route・DBは変更なし。</x:v>
+        <x:v>CHG-MENU-20260929-01：U-01対応。固定Menu Code・menus契約・下流Bindingを整合。既存権限・Route・DBは変更なし。 Menu Code正本化を確認。Menu欄のData Scope本文を正本参照へ統一。</x:v>
       </x:c>
       <x:c r="D22" t="str">
         <x:v>－</x:v>
@@ -2741,7 +2741,7 @@
         <x:v>×</x:v>
       </x:c>
       <x:c r="F9" s="33" t="str">
-        <x:v>PMは担当する未完了PJのACTIVE Memberかつ在籍社員のみ参照。更新系Menu/操作は非表示</x:v>
+        <x:v>Data Scopeは本書14_DataScope定義、API対応は13_API権限対応を参照。更新系Menu／操作は非表示。</x:v>
       </x:c>
       <x:c r="G9"/>
       <x:c r="H9"/>
@@ -2791,7 +2791,7 @@
         <x:v>○</x:v>
       </x:c>
       <x:c r="F11" s="33" t="str">
-        <x:v>担当・参加範囲</x:v>
+        <x:v>Data Scopeは本書14_DataScope定義、API対応は13_API権限対応を参照。</x:v>
       </x:c>
       <x:c r="G11"/>
       <x:c r="H11"/>
@@ -2843,7 +2843,7 @@
         <x:v>×</x:v>
       </x:c>
       <x:c r="F13" s="33" t="str">
-        <x:v>PMは担当PJ</x:v>
+        <x:v>Data Scopeは本書14_DataScope定義、API対応は13_API権限対応を参照。</x:v>
       </x:c>
       <x:c r="G13"/>
       <x:c r="H13"/>
@@ -2893,7 +2893,7 @@
         <x:v>○</x:v>
       </x:c>
       <x:c r="F15" s="33" t="str">
-        <x:v>参加PJのみ</x:v>
+        <x:v>Data Scopeは本書14_DataScope定義、API対応は13_API権限対応を参照。</x:v>
       </x:c>
       <x:c r="G15"/>
       <x:c r="H15"/>
@@ -2943,7 +2943,7 @@
         <x:v>×</x:v>
       </x:c>
       <x:c r="F17" s="33" t="str">
-        <x:v>PMは担当PJ</x:v>
+        <x:v>Data Scopeは本書14_DataScope定義、API対応は13_API権限対応を参照。</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="40" customHeight="1">
@@ -2989,7 +2989,7 @@
         <x:v>○</x:v>
       </x:c>
       <x:c r="F19" s="33" t="str">
-        <x:v>本人通知</x:v>
+        <x:v>Data Scopeは本書14_DataScope定義、API対応は13_API権限対応を参照。</x:v>
       </x:c>
     </x:row>
     <x:row r="20">

</xml_diff>